<commit_message>
feat(archery): 한 발 승부 쏘기 시간 5초 → 7.5초(노출 250 → 375틱)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#ArcheryRange.xlsx
+++ b/table/Datas/#ArcheryRange.xlsx
@@ -800,7 +800,7 @@
         <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -832,7 +832,7 @@
         <v>20</v>
       </c>
       <c r="F12" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>20</v>
       </c>
       <c r="F13" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -896,7 +896,7 @@
         <v>20</v>
       </c>
       <c r="F14" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G14" t="n">
         <v>1.7</v>
@@ -928,7 +928,7 @@
         <v>20</v>
       </c>
       <c r="F15" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -960,7 +960,7 @@
         <v>30</v>
       </c>
       <c r="F16" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -992,7 +992,7 @@
         <v>20</v>
       </c>
       <c r="F17" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G17" t="n">
         <v>2</v>
@@ -1024,7 +1024,7 @@
         <v>65</v>
       </c>
       <c r="F18" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1056,7 +1056,7 @@
         <v>30</v>
       </c>
       <c r="F19" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G19" t="n">
         <v>1.3</v>
@@ -1088,7 +1088,7 @@
         <v>20</v>
       </c>
       <c r="F20" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -1120,7 +1120,7 @@
         <v>45</v>
       </c>
       <c r="F21" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1152,7 +1152,7 @@
         <v>45</v>
       </c>
       <c r="F22" t="n">
-        <v>250</v>
+        <v>375</v>
       </c>
       <c r="G22" t="n">
         <v>1.3</v>

</xml_diff>